<commit_message>
feat: functioning LTN autoencoder
</commit_message>
<xml_diff>
--- a/.out/plots/isj-2019/table.xlsx
+++ b/.out/plots/isj-2019/table.xlsx
@@ -478,22 +478,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>P2P</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>p2p-0.3-1</t>
+          <t>medium-0.3-1</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.2434337677464752</v>
+        <v>0.1572370704616453</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5997234161552547</v>
+        <v>0.4988986784140969</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1527101837954875</v>
+        <v>0.09332509270704574</v>
       </c>
     </row>
     <row r="3">
@@ -509,22 +509,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>P2P</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>p2p-0.3-1</t>
+          <t>medium-0.3-1</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.1150453264294374</v>
+        <v>0.1552384267316394</v>
       </c>
       <c r="F3" t="n">
-        <v>0.06417537084552963</v>
+        <v>0.5</v>
       </c>
       <c r="G3" t="n">
-        <v>0.5548926014319809</v>
+        <v>0.09188298310671611</v>
       </c>
     </row>
     <row r="4">
@@ -540,22 +540,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>P2P</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>p2p-0.3-1</t>
+          <t>medium-0.3-1</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.3935342705887234</v>
+        <v>0.2726544530781608</v>
       </c>
       <c r="F4" t="n">
-        <v>0.7415094339622641</v>
+        <v>0.5197368421052632</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2678416702196427</v>
+        <v>0.1848004831849603</v>
       </c>
     </row>
     <row r="5">
@@ -571,22 +571,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>P2P</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>p2p-0.3-1</t>
+          <t>medium-0.3-1</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.3138019844243859</v>
+        <v>0.3095217376736166</v>
       </c>
       <c r="F5" t="n">
-        <v>0.2023526717557252</v>
+        <v>0.592948717948718</v>
       </c>
       <c r="G5" t="n">
-        <v>0.6985294117647058</v>
+        <v>0.2094199073557128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Add AxiomBuilder for building Declare Constraints
</commit_message>
<xml_diff>
--- a/.out/plots/isj-2019/table.xlsx
+++ b/.out/plots/isj-2019/table.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,22 +478,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>P2P</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>medium-0.3-1</t>
+          <t>p2p-0.3-1</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.1572370704616453</v>
+        <v>0.4215240253029719</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4988986784140969</v>
+        <v>0.4903259611088539</v>
       </c>
       <c r="G2" t="n">
-        <v>0.09332509270704574</v>
+        <v>0.3696545530595674</v>
       </c>
     </row>
     <row r="3">
@@ -509,53 +509,53 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>P2P</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>medium-0.3-1</t>
+          <t>p2p-0.3-1</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.1552384267316394</v>
+        <v>0.4052780134830651</v>
       </c>
       <c r="F3" t="n">
-        <v>0.5</v>
+        <v>0.4671488724033578</v>
       </c>
       <c r="G3" t="n">
-        <v>0.09188298310671611</v>
+        <v>0.3578792165932633</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Case</t>
+          <t>Attribute</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DAE</t>
+          <t>DAELTNFROZEN</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>P2P</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>medium-0.3-1</t>
+          <t>p2p-0.3-1</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.2726544530781608</v>
+        <v>0.4078022880014309</v>
       </c>
       <c r="F4" t="n">
-        <v>0.5197368421052632</v>
+        <v>0.4660778001542223</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1848004831849603</v>
+        <v>0.3624800088576139</v>
       </c>
     </row>
     <row r="5">
@@ -566,27 +566,89 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>DAE</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>P2P</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>p2p-0.3-1</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0.590826676593335</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.6592009807551822</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.5353034012295589</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Case</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>DAELTN</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>medium-0.3-1</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>0.3095217376736166</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.592948717948718</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.2094199073557128</v>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>P2P</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>p2p-0.3-1</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0.589639469547779</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.6545577385597573</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.5364363421309604</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Case</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DAELTNFROZEN</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>P2P</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>p2p-0.3-1</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0.5912273055607434</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.6495177217537605</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.5425377188518615</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: explore paper dataset
</commit_message>
<xml_diff>
--- a/.out/plots/isj-2019/table.xlsx
+++ b/.out/plots/isj-2019/table.xlsx
@@ -487,13 +487,13 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.4215240253029719</v>
+        <v>0.3843188140906739</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4903259611088539</v>
+        <v>0.3455646925633441</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3696545530595674</v>
+        <v>0.4328632236793544</v>
       </c>
     </row>
     <row r="3">
@@ -518,13 +518,13 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.4052780134830651</v>
+        <v>0.2767761993624065</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4671488724033578</v>
+        <v>0.4781789824365076</v>
       </c>
       <c r="G3" t="n">
-        <v>0.3578792165932633</v>
+        <v>0.1947500184533622</v>
       </c>
     </row>
     <row r="4">
@@ -549,13 +549,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.4078022880014309</v>
+        <v>0.310321365236007</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4660778001542223</v>
+        <v>0.4457090122947469</v>
       </c>
       <c r="G4" t="n">
-        <v>0.3624800088576139</v>
+        <v>0.2380206923701498</v>
       </c>
     </row>
     <row r="5">
@@ -580,13 +580,13 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.590826676593335</v>
+        <v>0.6391886795017844</v>
       </c>
       <c r="F5" t="n">
-        <v>0.6592009807551822</v>
+        <v>0.605193400687674</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5353034012295589</v>
+        <v>0.6772304666547471</v>
       </c>
     </row>
     <row r="6">
@@ -611,13 +611,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.589639469547779</v>
+        <v>0.4690644187812781</v>
       </c>
       <c r="F6" t="n">
-        <v>0.6545577385597573</v>
+        <v>0.6388183509916536</v>
       </c>
       <c r="G6" t="n">
-        <v>0.5364363421309604</v>
+        <v>0.3705877195395343</v>
       </c>
     </row>
     <row r="7">
@@ -642,13 +642,13 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.5912273055607434</v>
+        <v>0.5314162188223432</v>
       </c>
       <c r="F7" t="n">
-        <v>0.6495177217537605</v>
+        <v>0.6450297228276468</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5425377188518615</v>
+        <v>0.4518319602800204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: first successful run
</commit_message>
<xml_diff>
--- a/.out/plots/isj-2019/table.xlsx
+++ b/.out/plots/isj-2019/table.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,22 +478,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>P2P</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>p2p-0.3-1</t>
+          <t>paper-0.3-1</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.3843188140906739</v>
+        <v>0.2907735327541757</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3455646925633441</v>
+        <v>0.5130472755203126</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4328632236793544</v>
+        <v>0.2028781512605042</v>
       </c>
     </row>
     <row r="3">
@@ -504,58 +504,58 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DAELTN</t>
+          <t>DAELTNFROZEN</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>P2P</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>p2p-0.3-1</t>
+          <t>paper-0.3-1</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.2767761993624065</v>
+        <v>0.2763944297344673</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4781789824365076</v>
+        <v>0.3256451147239602</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1947500184533622</v>
+        <v>0.2400840336134454</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Attribute</t>
+          <t>Case</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DAELTNFROZEN</t>
+          <t>DAE</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>P2P</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>p2p-0.3-1</t>
+          <t>paper-0.3-1</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.310321365236007</v>
+        <v>0.5082208774864756</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4457090122947469</v>
+        <v>0.6180976234855545</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2380206923701498</v>
+        <v>0.4315126050420168</v>
       </c>
     </row>
     <row r="5">
@@ -566,89 +566,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DAE</t>
+          <t>DAELTNFROZEN</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>P2P</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>p2p-0.3-1</t>
+          <t>paper-0.3-1</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.6391886795017844</v>
+        <v>0.6013561353390825</v>
       </c>
       <c r="F5" t="n">
-        <v>0.605193400687674</v>
+        <v>0.6001957577559718</v>
       </c>
       <c r="G5" t="n">
-        <v>0.6772304666547471</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Case</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>DAELTN</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>P2P</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>p2p-0.3-1</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>0.4690644187812781</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.6388183509916536</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.3705877195395343</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Case</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>DAELTNFROZEN</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>P2P</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>p2p-0.3-1</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>0.5314162188223432</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.6450297228276468</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.4518319602800204</v>
+        <v>0.6025210084033614</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: CArry out LTN dataset fraction-wise study on synthetic dataset
</commit_message>
<xml_diff>
--- a/.out/plots/isj-2019/table.xlsx
+++ b/.out/plots/isj-2019/table.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Attribute</t>
+          <t>Case</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -487,106 +487,13 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.2907735327541757</v>
+        <v>0.5231838720889816</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5130472755203126</v>
+        <v>0.6339285714285714</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2028781512605042</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>DAELTNFROZEN</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Paper</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>paper-0.3-1</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>0.2763944297344673</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.3256451147239602</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.2400840336134454</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Case</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>DAE</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Paper</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>paper-0.3-1</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>0.5082208774864756</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.6180976234855545</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.4315126050420168</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Case</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>DAELTNFROZEN</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Paper</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>paper-0.3-1</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>0.6013561353390825</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.6001957577559718</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.6025210084033614</v>
+        <v>0.4453781512605042</v>
       </c>
     </row>
   </sheetData>

</xml_diff>